<commit_message>
just some data files
</commit_message>
<xml_diff>
--- a/data/zone-10.xlsx
+++ b/data/zone-10.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">timezon</t>
   </si>
   <si>
-    <t xml:space="preserve">Etc/GMT-6</t>
+    <t xml:space="preserve">Etc/GMT+11</t>
   </si>
   <si>
     <t xml:space="preserve">location</t>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t xml:space="preserve">COURSEFORBOYS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COURSEFORGIRLS</t>
   </si>
   <si>
     <t xml:space="preserve">action</t>
@@ -388,7 +391,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="17.11"/>
@@ -449,6 +452,17 @@
       </c>
       <c r="C5" s="2" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -475,13 +489,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
testx +zone-10 OK with no confirmation
</commit_message>
<xml_diff>
--- a/data/zone-10.xlsx
+++ b/data/zone-10.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">timezon</t>
   </si>
   <si>
-    <t xml:space="preserve">Etc/GMT-12</t>
+    <t xml:space="preserve">Etc/GMT-11</t>
   </si>
   <si>
     <t xml:space="preserve">location</t>
@@ -45,7 +45,7 @@
     <t xml:space="preserve">targets</t>
   </si>
   <si>
-    <t xml:space="preserve">CC MA MA-D FA KDB DH1</t>
+    <t xml:space="preserve">CC</t>
   </si>
   <si>
     <t xml:space="preserve">default_period</t>
@@ -75,31 +75,37 @@
     <t xml:space="preserve">ServicePeriod</t>
   </si>
   <si>
-    <t xml:space="preserve">WORKPERIOD</t>
+    <t xml:space="preserve">INBETWEEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">container</t>
+  </si>
+  <si>
+    <t xml:space="preserve">after</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service d0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Children / teens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert1</t>
   </si>
   <si>
     <t xml:space="preserve">Service</t>
   </si>
   <si>
-    <t xml:space="preserve">SITSERVE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Children / teens (3d)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Child-Teen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COURSEFORBOYS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COURSEFORGIRLS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">container</t>
+    <t xml:space="preserve">Service after d0</t>
   </si>
 </sst>
 </file>
@@ -109,7 +115,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -130,12 +136,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -180,12 +180,8 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -193,7 +189,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -217,37 +213,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -322,56 +318,52 @@
   </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.37"/>
-  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>1370</v>
+      <c r="B3" s="1" t="n">
+        <v>1396</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>1</v>
+      <c r="B4" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -391,78 +383,45 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="17.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -481,27 +440,84 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="13.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="C3" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>